<commit_message>
Add human-related features interaction to XGBoost dataset. Add app layout V2.
</commit_message>
<xml_diff>
--- a/Documents/FireComparision.xlsx
+++ b/Documents/FireComparision.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Master\ForestFlameAlert\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E329A9EE-5330-4FF8-94CB-876B327E2079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A6BE87-69C8-444E-873A-24A21C8BE181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6B87C76C-D74B-4D7A-9F6C-EB31A7D3D443}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6B87C76C-D74B-4D7A-9F6C-EB31A7D3D443}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="95">
   <si>
     <t>=============================================</t>
   </si>
@@ -253,14 +254,79 @@
   </si>
   <si>
     <t xml:space="preserve">  ndii                   -0.039428</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  fire_prob  : 0.083140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  dist_road_km           29.122931</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  dist_settlement_km     31.347641</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  dist_forest_edge_km    0.000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  dist_powerline_km      65.761856</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  lulc_class             10.000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  cropland_frac_1km      0.000920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  tree_cover_pct         77.462784</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  deforestation_lag_1y   1.620000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  nightlight_mean        0.000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  pop_density            86.278778</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  fire_count_prev_year   1.000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  fire_count_prev_3y     1.000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  fire_freq_5y           0.800000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  days_since_last_fire   133.000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  burn_season_flag       1.000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  days_since_harvest     14.000000</t>
+  </si>
+  <si>
+    <t>Veg_Index</t>
+  </si>
+  <si>
+    <t>Veg_Index + Human features</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -288,8 +354,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1030,4 +1097,407 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6EF787A-D3EB-4F18-9AEC-5FEDDC2B41BE}">
+  <dimension ref="A1:B55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="46.21875" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B40" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B44" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B46" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B48" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B50" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B52" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B53" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B54" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B55" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>